<commit_message>
feat(uiux & settings): add classroom name edit option, settings page, notification drawer, and modern card UI
</commit_message>
<xml_diff>
--- a/data/master_academic_plan.xlsx
+++ b/data/master_academic_plan.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6096,6 +6096,561 @@
         <v>0</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-001</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Unit III — Database Design and Normalization</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Introduction to Database Normalization: First Normal Form (1NF)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-002</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Unit III — Database Design and Normalization</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Second Normal Form (2NF) and Third Normal Form (3NF) Principles</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-003</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Unit III — Database Design and Normalization</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Boyce-Codd Normal Form (BCNF) and Higher Normal Forms</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-004</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Unit III — Database Design and Normalization</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Practical: Database Schema Normalization and Denormalization Techniques</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-005</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Unit IV — Transaction Management and Concurrency Control</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>SQL Transactions: ACID Properties and Transaction Control Language (TCL)</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-006</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Unit IV — Transaction Management and Concurrency Control</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Concurrency Control: Locking Mechanisms and Deadlock Prevention</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-007</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Unit IV — Transaction Management and Concurrency Control</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Practical: Implementing SQL Transactions with COMMIT, ROLLBACK, and SAVEPOINT</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-008</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Unit IV — Transaction Management and Concurrency Control</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Isolation Levels and Anomalies: Dirty Reads, Phantom Reads, and Non-Repeatable Reads</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-009</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Unit IV — Transaction Management and Concurrency Control</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Case Study: Real-World Transaction Scenarios and Performance Optimization</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CSE-DMS-CSEB-010</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Database Management Systems</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Unit III-IV — Integrated Assessment</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Comprehensive Practical: Database Design, Normalization, and Transaction Implementation</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>CSE-B</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CSE-DSA-L6-0001</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Data Structures</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Unit III — Linked Lists</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Singly Linked List Implementation</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>CSE-C</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>